<commit_message>
Pre-launch: all changes, API key rotation required in next step
</commit_message>
<xml_diff>
--- a/exports/appointments.xlsx
+++ b/exports/appointments.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="All Appointments" sheetId="1" r:id="rId1"/>
-    <sheet name="Today (2026-04-25)" sheetId="2" r:id="rId2"/>
+    <sheet name="Today (2026-04-28)" sheetId="2" r:id="rId2"/>
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -455,13 +455,13 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-59-31</v>
+        <v>2026-07-24</v>
       </c>
       <c r="C2" t="str">
-        <v>09:00</v>
+        <v>11:00</v>
       </c>
       <c r="D2" t="str">
         <v>SCHEDULED</v>
@@ -470,7 +470,7 @@
         <v>Unknown</v>
       </c>
       <c r="F2" t="str">
-        <v>27619434732</v>
+        <v>150852404793537</v>
       </c>
       <c r="G2" t="str">
         <v/>
@@ -488,50 +488,12 @@
         <v/>
       </c>
       <c r="L2" t="str">
-        <v>2026/04/26, 00:33:53</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2026-04-27</v>
-      </c>
-      <c r="C3" t="str">
-        <v>15:00</v>
-      </c>
-      <c r="D3" t="str">
-        <v>SCHEDULED</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="F3" t="str">
-        <v>150852404793537</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Consultation</v>
-      </c>
-      <c r="I3">
-        <v>30</v>
-      </c>
-      <c r="J3" t="str">
-        <v>0.00</v>
-      </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v>2026/04/25, 19:13:34</v>
+        <v>2026/04/28, 05:52:40</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -617,7 +579,7 @@
         <v>Generated</v>
       </c>
       <c r="B2" t="str">
-        <v>2026/04/26, 00:33:53</v>
+        <v>2026/04/28, 05:52:40</v>
       </c>
     </row>
     <row r="4">
@@ -633,7 +595,7 @@
         <v>Scheduled</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -665,7 +627,7 @@
         <v>Total</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">

</xml_diff>